<commit_message>
demo-at: build triggered by rockphotog for commit 209d48145fcaaaa5a40875e1862c9451f8c83aad 209d48145fcaaaa5a40875e1862c9451f8c83aad
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
+++ b/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>0.1.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -66,13 +66,13 @@
     <t>Publisher</t>
   </si>
   <si>
-    <t>HL7 Norge</t>
+    <t>Helsedirektoratet</t>
   </si>
   <si>
     <t>Contact</t>
   </si>
   <si>
-    <t>HL7 Norge (https://www.hl7.no)</t>
+    <t>Helsedirektoratet (https://www.helsedirektoratet.no)</t>
   </si>
   <si>
     <t>Jurisdiction</t>
@@ -4601,10 +4601,10 @@
       <c r="M28" t="s" s="2">
         <v>271</v>
       </c>
-      <c r="N28" t="s" s="2">
+      <c r="N28" s="2"/>
+      <c r="O28" t="s" s="2">
         <v>272</v>
       </c>
-      <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>79</v>
       </c>

</xml_diff>

<commit_message>
demo-at: build triggered by rockphotog for commit 890085fa61e819516484950c814180ec1b3a7226 890085fa61e819516484950c814180ec1b3a7226
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
+++ b/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1706" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1705" uniqueCount="379">
   <si>
     <t>Property</t>
   </si>
@@ -779,10 +779,7 @@
 The 'substanceExposureRisk' extension is available as a structured and more flexible alternative to the 'code' element for making positive or negative allergy or intolerance statements.  This extension provides the capability to make "no known allergy" (or "no risk of adverse reaction") statements regarding any coded substance/product (including cases when a pre-coordinated "no allergy to x" concept for that substance/product does not exist).  If the 'substanceExposureRisk' extension is present, the AllergyIntolerance.code element SHALL be omitted.</t>
   </si>
   <si>
-    <t>Type of the substance/product, allergy or intolerance condition or a code for absent/unknown allergy.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/uv/ips/ValueSet/allergies-intolerances-uv-ips</t>
+    <t>http://hl7.no/fhir/ig/demo-at/ValueSet/annen-allergi-som-kritisk-informasjon-7514</t>
   </si>
   <si>
     <t>substance/product:@@ -1561,7 +1558,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="106.67578125" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="50.62109375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="64.96484375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
@@ -4083,11 +4080,9 @@
       <c r="X23" t="s" s="2">
         <v>111</v>
       </c>
-      <c r="Y23" t="s" s="2">
+      <c r="Y23" s="2"/>
+      <c r="Z23" t="s" s="2">
         <v>242</v>
-      </c>
-      <c r="Z23" t="s" s="2">
-        <v>243</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>79</v>
@@ -4120,25 +4115,25 @@
         <v>99</v>
       </c>
       <c r="AK23" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="AL23" t="s" s="2">
         <v>244</v>
       </c>
-      <c r="AL23" t="s" s="2">
+      <c r="AM23" t="s" s="2">
         <v>245</v>
-      </c>
-      <c r="AM23" t="s" s="2">
-        <v>246</v>
       </c>
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
@@ -4157,13 +4152,13 @@
         <v>88</v>
       </c>
       <c r="K24" t="s" s="2">
+        <v>248</v>
+      </c>
+      <c r="L24" t="s" s="2">
         <v>249</v>
       </c>
-      <c r="L24" t="s" s="2">
+      <c r="M24" t="s" s="2">
         <v>250</v>
-      </c>
-      <c r="M24" t="s" s="2">
-        <v>251</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -4214,7 +4209,7 @@
         <v>79</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>87</v>
@@ -4229,21 +4224,21 @@
         <v>99</v>
       </c>
       <c r="AK24" t="s" s="2">
+        <v>251</v>
+      </c>
+      <c r="AL24" t="s" s="2">
         <v>252</v>
       </c>
-      <c r="AL24" t="s" s="2">
+      <c r="AM24" t="s" s="2">
         <v>253</v>
-      </c>
-      <c r="AM24" t="s" s="2">
-        <v>254</v>
       </c>
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4266,13 +4261,13 @@
         <v>79</v>
       </c>
       <c r="K25" t="s" s="2">
+        <v>255</v>
+      </c>
+      <c r="L25" t="s" s="2">
         <v>256</v>
       </c>
-      <c r="L25" t="s" s="2">
+      <c r="M25" t="s" s="2">
         <v>257</v>
-      </c>
-      <c r="M25" t="s" s="2">
-        <v>258</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -4323,7 +4318,7 @@
         <v>79</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>77</v>
@@ -4338,10 +4333,10 @@
         <v>99</v>
       </c>
       <c r="AK25" t="s" s="2">
+        <v>258</v>
+      </c>
+      <c r="AL25" t="s" s="2">
         <v>259</v>
-      </c>
-      <c r="AL25" t="s" s="2">
-        <v>260</v>
       </c>
       <c r="AM25" t="s" s="2">
         <v>79</v>
@@ -4349,10 +4344,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4378,10 +4373,10 @@
         <v>165</v>
       </c>
       <c r="L26" t="s" s="2">
+        <v>261</v>
+      </c>
+      <c r="M26" t="s" s="2">
         <v>262</v>
-      </c>
-      <c r="M26" t="s" s="2">
-        <v>263</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
@@ -4430,7 +4425,7 @@
         <v>136</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>77</v>
@@ -4445,10 +4440,10 @@
         <v>99</v>
       </c>
       <c r="AK26" t="s" s="2">
+        <v>263</v>
+      </c>
+      <c r="AL26" t="s" s="2">
         <v>264</v>
-      </c>
-      <c r="AL26" t="s" s="2">
-        <v>265</v>
       </c>
       <c r="AM26" t="s" s="2">
         <v>79</v>
@@ -4456,13 +4451,13 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
+        <v>265</v>
+      </c>
+      <c r="B27" t="s" s="2">
+        <v>260</v>
+      </c>
+      <c r="C27" t="s" s="2">
         <v>266</v>
-      </c>
-      <c r="B27" t="s" s="2">
-        <v>261</v>
-      </c>
-      <c r="C27" t="s" s="2">
-        <v>267</v>
       </c>
       <c r="D27" t="s" s="2">
         <v>79</v>
@@ -4487,10 +4482,10 @@
         <v>173</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -4541,7 +4536,7 @@
         <v>79</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>77</v>
@@ -4556,10 +4551,10 @@
         <v>99</v>
       </c>
       <c r="AK27" t="s" s="2">
+        <v>263</v>
+      </c>
+      <c r="AL27" t="s" s="2">
         <v>264</v>
-      </c>
-      <c r="AL27" t="s" s="2">
-        <v>265</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>79</v>
@@ -4567,10 +4562,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4596,14 +4591,14 @@
         <v>173</v>
       </c>
       <c r="L28" t="s" s="2">
+        <v>269</v>
+      </c>
+      <c r="M28" t="s" s="2">
         <v>270</v>
-      </c>
-      <c r="M28" t="s" s="2">
-        <v>271</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" t="s" s="2">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="P28" t="s" s="2">
         <v>79</v>
@@ -4652,7 +4647,7 @@
         <v>79</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>77</v>
@@ -4667,25 +4662,25 @@
         <v>99</v>
       </c>
       <c r="AK28" t="s" s="2">
+        <v>272</v>
+      </c>
+      <c r="AL28" t="s" s="2">
         <v>273</v>
       </c>
-      <c r="AL28" t="s" s="2">
+      <c r="AM28" t="s" s="2">
         <v>274</v>
-      </c>
-      <c r="AM28" t="s" s="2">
-        <v>275</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
@@ -4704,13 +4699,13 @@
         <v>79</v>
       </c>
       <c r="K29" t="s" s="2">
+        <v>277</v>
+      </c>
+      <c r="L29" t="s" s="2">
         <v>278</v>
       </c>
-      <c r="L29" t="s" s="2">
+      <c r="M29" t="s" s="2">
         <v>279</v>
-      </c>
-      <c r="M29" t="s" s="2">
-        <v>280</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -4761,7 +4756,7 @@
         <v>79</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>77</v>
@@ -4776,10 +4771,10 @@
         <v>99</v>
       </c>
       <c r="AK29" t="s" s="2">
+        <v>280</v>
+      </c>
+      <c r="AL29" t="s" s="2">
         <v>281</v>
-      </c>
-      <c r="AL29" t="s" s="2">
-        <v>282</v>
       </c>
       <c r="AM29" t="s" s="2">
         <v>79</v>
@@ -4787,14 +4782,14 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
@@ -4813,16 +4808,16 @@
         <v>88</v>
       </c>
       <c r="K30" t="s" s="2">
+        <v>284</v>
+      </c>
+      <c r="L30" t="s" s="2">
         <v>285</v>
       </c>
-      <c r="L30" t="s" s="2">
+      <c r="M30" t="s" s="2">
         <v>286</v>
       </c>
-      <c r="M30" t="s" s="2">
+      <c r="N30" t="s" s="2">
         <v>287</v>
-      </c>
-      <c r="N30" t="s" s="2">
-        <v>288</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -4872,7 +4867,7 @@
         <v>79</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>77</v>
@@ -4887,21 +4882,21 @@
         <v>99</v>
       </c>
       <c r="AK30" t="s" s="2">
+        <v>288</v>
+      </c>
+      <c r="AL30" t="s" s="2">
         <v>289</v>
       </c>
-      <c r="AL30" t="s" s="2">
+      <c r="AM30" t="s" s="2">
         <v>290</v>
-      </c>
-      <c r="AM30" t="s" s="2">
-        <v>291</v>
       </c>
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4927,13 +4922,13 @@
         <v>173</v>
       </c>
       <c r="L31" t="s" s="2">
+        <v>292</v>
+      </c>
+      <c r="M31" t="s" s="2">
         <v>293</v>
       </c>
-      <c r="M31" t="s" s="2">
+      <c r="N31" t="s" s="2">
         <v>294</v>
-      </c>
-      <c r="N31" t="s" s="2">
-        <v>295</v>
       </c>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
@@ -4983,7 +4978,7 @@
         <v>79</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>77</v>
@@ -4998,7 +4993,7 @@
         <v>99</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>79</v>
@@ -5009,10 +5004,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5035,16 +5030,16 @@
         <v>79</v>
       </c>
       <c r="K32" t="s" s="2">
+        <v>297</v>
+      </c>
+      <c r="L32" t="s" s="2">
         <v>298</v>
       </c>
-      <c r="L32" t="s" s="2">
+      <c r="M32" t="s" s="2">
         <v>299</v>
       </c>
-      <c r="M32" t="s" s="2">
+      <c r="N32" t="s" s="2">
         <v>300</v>
-      </c>
-      <c r="N32" t="s" s="2">
-        <v>301</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -5094,7 +5089,7 @@
         <v>79</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>77</v>
@@ -5109,7 +5104,7 @@
         <v>99</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="AL32" t="s" s="2">
         <v>79</v>
@@ -5120,10 +5115,10 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5146,7 +5141,7 @@
         <v>79</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="L33" t="s" s="2">
         <v>147</v>
@@ -5229,10 +5224,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5258,10 +5253,10 @@
         <v>132</v>
       </c>
       <c r="L34" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="M34" t="s" s="2">
         <v>306</v>
-      </c>
-      <c r="M34" t="s" s="2">
-        <v>307</v>
       </c>
       <c r="N34" t="s" s="2">
         <v>179</v>
@@ -5340,10 +5335,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5366,16 +5361,16 @@
         <v>88</v>
       </c>
       <c r="K35" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="L35" t="s" s="2">
         <v>309</v>
       </c>
-      <c r="L35" t="s" s="2">
+      <c r="M35" t="s" s="2">
         <v>310</v>
       </c>
-      <c r="M35" t="s" s="2">
+      <c r="N35" t="s" s="2">
         <v>311</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>312</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5425,7 +5420,7 @@
         <v>79</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>77</v>
@@ -5440,7 +5435,7 @@
         <v>99</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>79</v>
@@ -5451,10 +5446,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5480,10 +5475,10 @@
         <v>173</v>
       </c>
       <c r="L36" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="M36" t="s" s="2">
         <v>316</v>
-      </c>
-      <c r="M36" t="s" s="2">
-        <v>317</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5534,7 +5529,7 @@
         <v>79</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>77</v>
@@ -5549,7 +5544,7 @@
         <v>99</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>79</v>
@@ -5560,10 +5555,10 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5586,13 +5581,13 @@
         <v>88</v>
       </c>
       <c r="K37" t="s" s="2">
+        <v>320</v>
+      </c>
+      <c r="L37" t="s" s="2">
         <v>321</v>
       </c>
-      <c r="L37" t="s" s="2">
+      <c r="M37" t="s" s="2">
         <v>322</v>
-      </c>
-      <c r="M37" t="s" s="2">
-        <v>323</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -5643,7 +5638,7 @@
         <v>79</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>87</v>
@@ -5658,7 +5653,7 @@
         <v>99</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>79</v>
@@ -5669,10 +5664,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5695,13 +5690,13 @@
         <v>79</v>
       </c>
       <c r="K38" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="L38" t="s" s="2">
         <v>327</v>
       </c>
-      <c r="L38" t="s" s="2">
+      <c r="M38" t="s" s="2">
         <v>328</v>
-      </c>
-      <c r="M38" t="s" s="2">
-        <v>329</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5752,7 +5747,7 @@
         <v>79</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>77</v>
@@ -5767,7 +5762,7 @@
         <v>99</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>79</v>
@@ -5778,10 +5773,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5804,7 +5799,7 @@
         <v>79</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="L39" t="s" s="2">
         <v>147</v>
@@ -5887,10 +5882,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5916,10 +5911,10 @@
         <v>132</v>
       </c>
       <c r="L40" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="M40" t="s" s="2">
         <v>306</v>
-      </c>
-      <c r="M40" t="s" s="2">
-        <v>307</v>
       </c>
       <c r="N40" t="s" s="2">
         <v>179</v>
@@ -5998,14 +5993,14 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
@@ -6027,10 +6022,10 @@
         <v>132</v>
       </c>
       <c r="L41" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="M41" t="s" s="2">
         <v>335</v>
-      </c>
-      <c r="M41" t="s" s="2">
-        <v>336</v>
       </c>
       <c r="N41" t="s" s="2">
         <v>179</v>
@@ -6085,7 +6080,7 @@
         <v>79</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>77</v>
@@ -6111,10 +6106,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6140,13 +6135,13 @@
         <v>192</v>
       </c>
       <c r="L42" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="M42" t="s" s="2">
         <v>339</v>
       </c>
-      <c r="M42" t="s" s="2">
+      <c r="N42" t="s" s="2">
         <v>340</v>
-      </c>
-      <c r="N42" t="s" s="2">
-        <v>341</v>
       </c>
       <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
@@ -6172,11 +6167,11 @@
         <v>79</v>
       </c>
       <c r="X42" t="s" s="2">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="Y42" s="2"/>
       <c r="Z42" t="s" s="2">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="AA42" t="s" s="2">
         <v>79</v>
@@ -6194,7 +6189,7 @@
         <v>79</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>77</v>
@@ -6209,7 +6204,7 @@
         <v>99</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="AL42" t="s" s="2">
         <v>79</v>
@@ -6220,14 +6215,14 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
@@ -6249,13 +6244,13 @@
         <v>192</v>
       </c>
       <c r="L43" t="s" s="2">
+        <v>346</v>
+      </c>
+      <c r="M43" t="s" s="2">
         <v>347</v>
       </c>
-      <c r="M43" t="s" s="2">
+      <c r="N43" t="s" s="2">
         <v>348</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>349</v>
       </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
@@ -6284,11 +6279,11 @@
         <v>111</v>
       </c>
       <c r="Y43" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="Z43" t="s" s="2">
         <v>350</v>
       </c>
-      <c r="Z43" t="s" s="2">
-        <v>351</v>
-      </c>
       <c r="AA43" t="s" s="2">
         <v>79</v>
       </c>
@@ -6305,7 +6300,7 @@
         <v>79</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>87</v>
@@ -6326,19 +6321,19 @@
         <v>79</v>
       </c>
       <c r="AM43" t="s" s="2">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -6357,16 +6352,16 @@
         <v>79</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="L44" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="M44" t="s" s="2">
         <v>355</v>
       </c>
-      <c r="M44" t="s" s="2">
+      <c r="N44" t="s" s="2">
         <v>356</v>
-      </c>
-      <c r="N44" t="s" s="2">
-        <v>357</v>
       </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
@@ -6416,7 +6411,7 @@
         <v>79</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>77</v>
@@ -6431,7 +6426,7 @@
         <v>99</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>79</v>
@@ -6442,10 +6437,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6471,10 +6466,10 @@
         <v>173</v>
       </c>
       <c r="L45" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>360</v>
-      </c>
-      <c r="M45" t="s" s="2">
-        <v>361</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6525,7 +6520,7 @@
         <v>79</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>77</v>
@@ -6540,21 +6535,21 @@
         <v>99</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6580,13 +6575,13 @@
         <v>107</v>
       </c>
       <c r="L46" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="M46" t="s" s="2">
         <v>364</v>
       </c>
-      <c r="M46" t="s" s="2">
+      <c r="N46" t="s" s="2">
         <v>365</v>
-      </c>
-      <c r="N46" t="s" s="2">
-        <v>366</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6615,11 +6610,11 @@
         <v>196</v>
       </c>
       <c r="Y46" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="Z46" t="s" s="2">
         <v>367</v>
       </c>
-      <c r="Z46" t="s" s="2">
-        <v>368</v>
-      </c>
       <c r="AA46" t="s" s="2">
         <v>79</v>
       </c>
@@ -6636,7 +6631,7 @@
         <v>79</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>77</v>
@@ -6662,10 +6657,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -6691,13 +6686,13 @@
         <v>192</v>
       </c>
       <c r="L47" t="s" s="2">
+        <v>369</v>
+      </c>
+      <c r="M47" t="s" s="2">
         <v>370</v>
       </c>
-      <c r="M47" t="s" s="2">
+      <c r="N47" t="s" s="2">
         <v>371</v>
-      </c>
-      <c r="N47" t="s" s="2">
-        <v>372</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -6723,14 +6718,14 @@
         <v>79</v>
       </c>
       <c r="X47" t="s" s="2">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="Y47" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="Z47" t="s" s="2">
         <v>373</v>
       </c>
-      <c r="Z47" t="s" s="2">
-        <v>374</v>
-      </c>
       <c r="AA47" t="s" s="2">
         <v>79</v>
       </c>
@@ -6747,7 +6742,7 @@
         <v>79</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>77</v>
@@ -6762,7 +6757,7 @@
         <v>99</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="AL47" t="s" s="2">
         <v>79</v>
@@ -6773,10 +6768,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -6799,16 +6794,16 @@
         <v>79</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="L48" t="s" s="2">
+        <v>376</v>
+      </c>
+      <c r="M48" t="s" s="2">
         <v>377</v>
       </c>
-      <c r="M48" t="s" s="2">
+      <c r="N48" t="s" s="2">
         <v>378</v>
-      </c>
-      <c r="N48" t="s" s="2">
-        <v>379</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
@@ -6858,7 +6853,7 @@
         <v>79</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>77</v>
@@ -6873,7 +6868,7 @@
         <v>99</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="AL48" t="s" s="2">
         <v>79</v>

</xml_diff>

<commit_message>
demo-at: build triggered by rockphotog for commit 582d2df4853f98c0847d4d927ce18fef13dbd91d 582d2df4853f98c0847d4d927ce18fef13dbd91d
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
+++ b/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.1</t>
+    <t>0.1.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -775,7 +775,7 @@
     <t>Merk: Det vil bli endringer i anbefaling til koding av legemidler og substanser (agens) når ny standard for identifisering av legemidler implementeres i Norge (IDMP).</t>
   </si>
   <si>
-    <t>http://hl7.no/fhir/ig/demo-at/ValueSet/allergener-7852</t>
+    <t>http://hl7.no/fhir/ig/demo-at/ValueSet/annen-allergi-som-kritisk-informasjon-7514</t>
   </si>
   <si>
     <t>substance/product:@@ -1541,7 +1541,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="106.67578125" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="50.62109375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="64.96484375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>

</xml_diff>

<commit_message>
demo-at: build triggered by rockphotog for commit f7f422ac3b72696bf4858aa981d7ea19aa25c818 f7f422ac3b72696bf4858aa981d7ea19aa25c818
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
+++ b/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
@@ -9,11 +9,14 @@
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AM$48</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1706" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1707" uniqueCount="383">
   <si>
     <t>Property</t>
   </si>
@@ -30,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.2</t>
+    <t>0.1.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -851,6 +854,9 @@
     <t>Estimated or actual date,  date-time, or age when allergy or intolerance was identified.</t>
   </si>
   <si>
+    <t>closed</t>
+  </si>
+  <si>
     <t>effectiveTime.low</t>
   </si>
   <si>
@@ -863,7 +869,13 @@
     <t>onsetDateTime</t>
   </si>
   <si>
-    <t>Onset date</t>
+    <t>Starttidspunkt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tidspunkt da overfølsomheten eller den uønskede reaksjonen ble konstatert. Tidspunkt kan være spesifikk (dag-tidspunkt) eller uspesifikk (årstall, tiår). </t>
+  </si>
+  <si>
+    <t>EHDS krever dato/tid, alder må konverteres.</t>
   </si>
   <si>
     <t>AllergyIntolerance.recordedDate</t>
@@ -872,7 +884,7 @@
     <t>Registreringsdato</t>
   </si>
   <si>
-    <t xml:space="preserve">Tidspunkt da overfølsomheten eller den uønskede reaksjonen ble konstatert. Tidspunkt kan være spesifikk (dag-tidspunkt) eller uspesifikk (årstall, tiår). </t>
+    <t>The recordedDate represents when this particular AllergyIntolerance record was created in the system, which is often a system-generated date.</t>
   </si>
   <si>
     <t>Obligatorisk i Kjernejournal</t>
@@ -1338,6 +1350,21 @@
       <alignment vertical="top" wrapText="true"/>
     </xf>
   </cellXfs>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor indexed="22"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color indexed="22"/>
+        <i val="true"/>
+      </font>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -1675,7 +1702,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" hidden="true">
       <c r="A2" t="s" s="2">
         <v>31</v>
       </c>
@@ -1786,7 +1813,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" hidden="true">
       <c r="A3" t="s" s="2">
         <v>87</v>
       </c>
@@ -1897,7 +1924,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" hidden="true">
       <c r="A4" t="s" s="2">
         <v>95</v>
       </c>
@@ -2006,7 +2033,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" hidden="true">
       <c r="A5" t="s" s="2">
         <v>101</v>
       </c>
@@ -2117,7 +2144,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" hidden="true">
       <c r="A6" t="s" s="2">
         <v>107</v>
       </c>
@@ -2228,7 +2255,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" hidden="true">
       <c r="A7" t="s" s="2">
         <v>116</v>
       </c>
@@ -2339,7 +2366,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" hidden="true">
       <c r="A8" t="s" s="2">
         <v>124</v>
       </c>
@@ -2450,7 +2477,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" hidden="true">
       <c r="A9" t="s" s="2">
         <v>132</v>
       </c>
@@ -2557,7 +2584,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
         <v>140</v>
       </c>
@@ -2670,7 +2697,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
         <v>146</v>
       </c>
@@ -2779,7 +2806,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
         <v>153</v>
       </c>
@@ -2888,7 +2915,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
         <v>157</v>
       </c>
@@ -2999,7 +3026,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
         <v>164</v>
       </c>
@@ -3106,7 +3133,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
         <v>172</v>
       </c>
@@ -3217,7 +3244,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
         <v>176</v>
       </c>
@@ -3330,7 +3357,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
         <v>183</v>
       </c>
@@ -3462,7 +3489,7 @@
         <v>88</v>
       </c>
       <c r="H18" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I18" t="s" s="2">
         <v>89</v>
@@ -3573,7 +3600,7 @@
         <v>88</v>
       </c>
       <c r="H19" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I19" t="s" s="2">
         <v>89</v>
@@ -3665,7 +3692,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
         <v>209</v>
       </c>
@@ -3776,7 +3803,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
         <v>219</v>
       </c>
@@ -3887,7 +3914,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
         <v>228</v>
       </c>
@@ -4017,7 +4044,7 @@
         <v>88</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>80</v>
@@ -4107,7 +4134,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
         <v>247</v>
       </c>
@@ -4216,7 +4243,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
         <v>255</v>
       </c>
@@ -4325,7 +4352,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
         <v>261</v>
       </c>
@@ -4405,7 +4432,7 @@
         <v>80</v>
       </c>
       <c r="AE26" t="s" s="2">
-        <v>137</v>
+        <v>264</v>
       </c>
       <c r="AF26" t="s" s="2">
         <v>261</v>
@@ -4423,24 +4450,24 @@
         <v>100</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AM26" t="s" s="2">
         <v>80</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B27" t="s" s="2">
         <v>261</v>
       </c>
       <c r="C27" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D27" t="s" s="2">
         <v>80</v>
@@ -4465,13 +4492,15 @@
         <v>174</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="N27" s="2"/>
-      <c r="O27" s="2"/>
+      <c r="O27" t="s" s="2">
+        <v>271</v>
+      </c>
       <c r="P27" t="s" s="2">
         <v>80</v>
       </c>
@@ -4534,21 +4563,21 @@
         <v>100</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>80</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4574,14 +4603,14 @@
         <v>174</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" t="s" s="2">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="P28" t="s" s="2">
         <v>80</v>
@@ -4630,7 +4659,7 @@
         <v>80</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -4645,25 +4674,25 @@
         <v>100</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
@@ -4682,13 +4711,13 @@
         <v>80</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -4739,7 +4768,7 @@
         <v>80</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
@@ -4754,25 +4783,25 @@
         <v>100</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="AM29" t="s" s="2">
         <v>80</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
@@ -4791,16 +4820,16 @@
         <v>89</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -4850,7 +4879,7 @@
         <v>80</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -4865,21 +4894,21 @@
         <v>100</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4905,13 +4934,13 @@
         <v>174</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
@@ -4961,7 +4990,7 @@
         <v>80</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -4976,7 +5005,7 @@
         <v>100</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>80</v>
@@ -4985,12 +5014,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5013,16 +5042,16 @@
         <v>80</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -5072,7 +5101,7 @@
         <v>80</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>78</v>
@@ -5087,7 +5116,7 @@
         <v>100</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="AL32" t="s" s="2">
         <v>80</v>
@@ -5096,12 +5125,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5124,7 +5153,7 @@
         <v>80</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="L33" t="s" s="2">
         <v>148</v>
@@ -5205,12 +5234,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5236,10 +5265,10 @@
         <v>133</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="N34" t="s" s="2">
         <v>180</v>
@@ -5316,12 +5345,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5344,16 +5373,16 @@
         <v>89</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5403,7 +5432,7 @@
         <v>80</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -5418,7 +5447,7 @@
         <v>100</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>80</v>
@@ -5427,12 +5456,12 @@
         <v>131</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5458,10 +5487,10 @@
         <v>174</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5512,7 +5541,7 @@
         <v>80</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -5527,7 +5556,7 @@
         <v>100</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>80</v>
@@ -5536,12 +5565,12 @@
         <v>131</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5564,13 +5593,13 @@
         <v>89</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -5621,7 +5650,7 @@
         <v>80</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>88</v>
@@ -5636,7 +5665,7 @@
         <v>100</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>80</v>
@@ -5645,12 +5674,12 @@
         <v>131</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5673,13 +5702,13 @@
         <v>80</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5730,7 +5759,7 @@
         <v>80</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -5745,7 +5774,7 @@
         <v>100</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>80</v>
@@ -5754,12 +5783,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5782,7 +5811,7 @@
         <v>80</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="L39" t="s" s="2">
         <v>148</v>
@@ -5863,12 +5892,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5894,10 +5923,10 @@
         <v>133</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="N40" t="s" s="2">
         <v>180</v>
@@ -5974,16 +6003,16 @@
         <v>80</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
@@ -6005,10 +6034,10 @@
         <v>133</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="N41" t="s" s="2">
         <v>180</v>
@@ -6063,7 +6092,7 @@
         <v>80</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6087,12 +6116,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6118,13 +6147,13 @@
         <v>193</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="N42" t="s" s="2">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
@@ -6150,11 +6179,11 @@
         <v>80</v>
       </c>
       <c r="X42" t="s" s="2">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="Y42" s="2"/>
       <c r="Z42" t="s" s="2">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="AA42" t="s" s="2">
         <v>80</v>
@@ -6172,7 +6201,7 @@
         <v>80</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>78</v>
@@ -6187,7 +6216,7 @@
         <v>100</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="AL42" t="s" s="2">
         <v>80</v>
@@ -6196,16 +6225,16 @@
         <v>80</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
@@ -6227,13 +6256,13 @@
         <v>193</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="N43" t="s" s="2">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
@@ -6262,10 +6291,10 @@
         <v>112</v>
       </c>
       <c r="Y43" t="s" s="2">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="Z43" t="s" s="2">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="AA43" t="s" s="2">
         <v>80</v>
@@ -6283,7 +6312,7 @@
         <v>80</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>88</v>
@@ -6304,19 +6333,19 @@
         <v>80</v>
       </c>
       <c r="AM43" t="s" s="2">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -6335,16 +6364,16 @@
         <v>80</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="N44" t="s" s="2">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
@@ -6394,7 +6423,7 @@
         <v>80</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>78</v>
@@ -6409,7 +6438,7 @@
         <v>100</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>80</v>
@@ -6418,12 +6447,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6449,10 +6478,10 @@
         <v>174</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6503,7 +6532,7 @@
         <v>80</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>78</v>
@@ -6518,21 +6547,21 @@
         <v>100</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6558,13 +6587,13 @@
         <v>108</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6593,10 +6622,10 @@
         <v>197</v>
       </c>
       <c r="Y46" t="s" s="2">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="Z46" t="s" s="2">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>80</v>
@@ -6614,7 +6643,7 @@
         <v>80</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
@@ -6638,12 +6667,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -6669,13 +6698,13 @@
         <v>193</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -6701,13 +6730,13 @@
         <v>80</v>
       </c>
       <c r="X47" t="s" s="2">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="Y47" t="s" s="2">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="Z47" t="s" s="2">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="AA47" t="s" s="2">
         <v>80</v>
@@ -6725,7 +6754,7 @@
         <v>80</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>78</v>
@@ -6740,7 +6769,7 @@
         <v>100</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="AL47" t="s" s="2">
         <v>80</v>
@@ -6749,12 +6778,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -6777,16 +6806,16 @@
         <v>80</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="N48" t="s" s="2">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
@@ -6836,7 +6865,7 @@
         <v>80</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>78</v>
@@ -6851,7 +6880,7 @@
         <v>100</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="AL48" t="s" s="2">
         <v>80</v>
@@ -6861,6 +6890,24 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AM48">
+    <filterColumn colId="7">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+    <filterColumn colId="27">
+      <filters blank="true"/>
+    </filterColumn>
+  </autoFilter>
+  <conditionalFormatting sqref="A2:AI47">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$G2&lt;&gt;"Y"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$Q2&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
demo-at: build triggered by rockphotog for commit eb4af79f6fb1ad772802b0d3e61950de0fbdc4eb eb4af79f6fb1ad772802b0d3e61950de0fbdc4eb
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
+++ b/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1707" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1707" uniqueCount="382">
   <si>
     <t>Property</t>
   </si>
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.3</t>
+    <t>0.1.4</t>
   </si>
   <si>
     <t>Name</t>
@@ -469,28 +469,32 @@
     <t>The date or estimated date that the allergy or intolerance resolved. This is called abatement because of the many overloaded connotations associated with resolution.</t>
   </si>
   <si>
-    <t>Age is generally used when the patient reports an age at which the allergy or intolerance abated. If there is no abatement element, the clinicalStatus can be used to convey whether allergy or intolerance has resolved or not. When abatementString exists, it conveys that the allergy or intolerance is abated.</t>
-  </si>
-  <si>
-    <t>AllergyIntolerance.extension:abatement.id</t>
-  </si>
-  <si>
-    <t>AllergyIntolerance.extension.id</t>
-  </si>
-  <si>
-    <t>Unique id for inter-element referencing</t>
-  </si>
-  <si>
-    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
-  </si>
-  <si>
-    <t>Element.id</t>
+    <t>Age is generally used when the patient reports an age at which the AllergyIntolerance was abated. Period is generally used to convey an imprecise abatement date that occurred within the time period. Range is generally used to convey an imprecise age range (e.g. 4 to 6 years old). If there is no abatement element, the clinicalStatus can be used to convey whether allergy or intolerance has resolved or not. When abatementString exists, it conveys that the allergy or intolerance is abated.</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1
 </t>
   </si>
   <si>
+    <t>AllergyIntolerance.extension:abatement.id</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.extension.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">string
+</t>
+  </si>
+  <si>
+    <t>Unique id for inter-element referencing</t>
+  </si>
+  <si>
+    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
+  </si>
+  <si>
+    <t>Element.id</t>
+  </si>
+  <si>
     <t>n/a</t>
   </si>
   <si>
@@ -540,7 +544,7 @@
     <t>Value of extension</t>
   </si>
   <si>
-    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R5/extensibility.html) for a list).</t>
+    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
   </si>
   <si>
     <t xml:space="preserve">type:$this}
@@ -550,10 +554,6 @@
     <t>Extension.value[x]</t>
   </si>
   <si>
-    <t xml:space="preserve">ext-1
-</t>
-  </si>
-  <si>
     <t>AllergyIntolerance.extension:abatement.value[x]:valueDateTime</t>
   </si>
   <si>
@@ -660,7 +660,7 @@
     <t>Assertion about certainty associated with the propensity, or potential risk, of a reaction to the identified substance (including pharmaceutical product).</t>
   </si>
   <si>
-    <t>The data type is CodeableConcept because verificationStatus has some clinical judgment involved, such that there might need to be more specificity than the required FHIR value set allows. For example, a SNOMED coding might allow for additional specificity.</t>
+    <t>Import need to handle missing verificationStatus</t>
   </si>
   <si>
     <t>Assertion about certainty associated with a propensity, or potential risk, of a reaction to the identified substance.</t>
@@ -744,7 +744,7 @@
     <t>Estimate of the potential clinical harm, or seriousness, of the reaction to the identified substance.</t>
   </si>
   <si>
-    <t>The default criticality value for any propensity to an adverse reaction should be 'Low Risk', indicating at the very least a relative contraindication to deliberate or voluntary exposure to the substance. 'High Risk' is flagged if the clinician has identified a propensity for a more serious or potentially life-threatening reaction, such as anaphylaxis, and implies an absolute contraindication to deliberate or voluntary exposure to the substance. If this element is missing, the criticality is unknown (though it may be known elsewhere).  Systems that capture a severity at the condition level are actually representing the concept of criticality whereas the severity documented at the reaction level is representing the true reaction severity.  Existing systems that are capturing both condition criticality and reaction severity may use the term "severity" to represent both.  Criticality is the worst it could be in the future (i.e. situation-agnostic) whereas severity is situation-dependent.</t>
+    <t>Import need to handle missing criticality</t>
   </si>
   <si>
     <t>Estimate of the potential clinical harm, or seriousness, of a reaction to an identified substance.</t>
@@ -986,10 +986,6 @@
   </si>
   <si>
     <t>AllergyIntolerance.note.id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">string
-</t>
   </si>
   <si>
     <t>AllergyIntolerance.note.extension</t>
@@ -2682,7 +2678,7 @@
         <v>79</v>
       </c>
       <c r="AI10" t="s" s="2">
-        <v>80</v>
+        <v>146</v>
       </c>
       <c r="AJ10" t="s" s="2">
         <v>139</v>
@@ -2699,10 +2695,10 @@
     </row>
     <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2725,13 +2721,13 @@
         <v>80</v>
       </c>
       <c r="K11" t="s" s="2">
-        <v>90</v>
+        <v>149</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -2782,7 +2778,7 @@
         <v>80</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>78</v>
@@ -2791,13 +2787,13 @@
         <v>88</v>
       </c>
       <c r="AI11" t="s" s="2">
-        <v>151</v>
+        <v>80</v>
       </c>
       <c r="AJ11" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AK11" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AL11" t="s" s="2">
         <v>80</v>
@@ -2808,10 +2804,10 @@
     </row>
     <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2882,7 +2878,7 @@
         <v>136</v>
       </c>
       <c r="AC12" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="AD12" t="s" s="2">
         <v>80</v>
@@ -2891,7 +2887,7 @@
         <v>137</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>78</v>
@@ -2917,10 +2913,10 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2946,13 +2942,13 @@
         <v>102</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2960,7 +2956,7 @@
       </c>
       <c r="Q13" s="2"/>
       <c r="R13" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="S13" t="s" s="2">
         <v>80</v>
@@ -3002,7 +2998,7 @@
         <v>80</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>88</v>
@@ -3028,10 +3024,10 @@
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -3054,13 +3050,13 @@
         <v>80</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -3099,7 +3095,7 @@
         <v>80</v>
       </c>
       <c r="AB14" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AC14" s="2"/>
       <c r="AD14" t="s" s="2">
@@ -3109,7 +3105,7 @@
         <v>137</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>78</v>
@@ -3118,7 +3114,7 @@
         <v>88</v>
       </c>
       <c r="AI14" t="s" s="2">
-        <v>171</v>
+        <v>80</v>
       </c>
       <c r="AJ14" t="s" s="2">
         <v>100</v>
@@ -3138,7 +3134,7 @@
         <v>172</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C15" t="s" s="2">
         <v>173</v>
@@ -3169,7 +3165,7 @@
         <v>175</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -3220,7 +3216,7 @@
         <v>80</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>78</v>
@@ -3229,7 +3225,7 @@
         <v>88</v>
       </c>
       <c r="AI15" t="s" s="2">
-        <v>171</v>
+        <v>80</v>
       </c>
       <c r="AJ15" t="s" s="2">
         <v>100</v>
@@ -3581,7 +3577,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
         <v>202</v>
       </c>
@@ -3594,13 +3590,13 @@
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G19" t="s" s="2">
         <v>88</v>
       </c>
       <c r="H19" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="I19" t="s" s="2">
         <v>89</v>
@@ -3927,7 +3923,7 @@
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="G22" t="s" s="2">
         <v>88</v>
@@ -4380,7 +4376,7 @@
         <v>80</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="L26" t="s" s="2">
         <v>262</v>
@@ -4425,7 +4421,7 @@
         <v>80</v>
       </c>
       <c r="AB26" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AC26" s="2"/>
       <c r="AD26" t="s" s="2">
@@ -5153,13 +5149,13 @@
         <v>80</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>307</v>
+        <v>149</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -5210,7 +5206,7 @@
         <v>80</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>78</v>
@@ -5225,7 +5221,7 @@
         <v>80</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AL33" t="s" s="2">
         <v>80</v>
@@ -5236,10 +5232,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5265,10 +5261,10 @@
         <v>133</v>
       </c>
       <c r="L34" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="M34" t="s" s="2">
         <v>309</v>
-      </c>
-      <c r="M34" t="s" s="2">
-        <v>310</v>
       </c>
       <c r="N34" t="s" s="2">
         <v>180</v>
@@ -5312,7 +5308,7 @@
         <v>136</v>
       </c>
       <c r="AC34" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="AD34" t="s" s="2">
         <v>80</v>
@@ -5321,7 +5317,7 @@
         <v>137</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>78</v>
@@ -5336,7 +5332,7 @@
         <v>139</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AL34" t="s" s="2">
         <v>80</v>
@@ -5347,10 +5343,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5373,16 +5369,16 @@
         <v>89</v>
       </c>
       <c r="K35" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="L35" t="s" s="2">
         <v>312</v>
       </c>
-      <c r="L35" t="s" s="2">
+      <c r="M35" t="s" s="2">
         <v>313</v>
       </c>
-      <c r="M35" t="s" s="2">
+      <c r="N35" t="s" s="2">
         <v>314</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>315</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5432,7 +5428,7 @@
         <v>80</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -5447,7 +5443,7 @@
         <v>100</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>80</v>
@@ -5458,10 +5454,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5487,10 +5483,10 @@
         <v>174</v>
       </c>
       <c r="L36" t="s" s="2">
+        <v>318</v>
+      </c>
+      <c r="M36" t="s" s="2">
         <v>319</v>
-      </c>
-      <c r="M36" t="s" s="2">
-        <v>320</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5541,7 +5537,7 @@
         <v>80</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -5556,7 +5552,7 @@
         <v>100</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>80</v>
@@ -5567,10 +5563,10 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5593,13 +5589,13 @@
         <v>89</v>
       </c>
       <c r="K37" t="s" s="2">
+        <v>323</v>
+      </c>
+      <c r="L37" t="s" s="2">
         <v>324</v>
       </c>
-      <c r="L37" t="s" s="2">
+      <c r="M37" t="s" s="2">
         <v>325</v>
-      </c>
-      <c r="M37" t="s" s="2">
-        <v>326</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -5650,7 +5646,7 @@
         <v>80</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>88</v>
@@ -5665,7 +5661,7 @@
         <v>100</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>80</v>
@@ -5676,10 +5672,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5702,13 +5698,13 @@
         <v>80</v>
       </c>
       <c r="K38" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="L38" t="s" s="2">
         <v>330</v>
       </c>
-      <c r="L38" t="s" s="2">
+      <c r="M38" t="s" s="2">
         <v>331</v>
-      </c>
-      <c r="M38" t="s" s="2">
-        <v>332</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5759,7 +5755,7 @@
         <v>80</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -5774,7 +5770,7 @@
         <v>100</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>80</v>
@@ -5785,10 +5781,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5811,13 +5807,13 @@
         <v>80</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>307</v>
+        <v>149</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -5868,7 +5864,7 @@
         <v>80</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
@@ -5883,7 +5879,7 @@
         <v>80</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>80</v>
@@ -5894,10 +5890,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5923,10 +5919,10 @@
         <v>133</v>
       </c>
       <c r="L40" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="M40" t="s" s="2">
         <v>309</v>
-      </c>
-      <c r="M40" t="s" s="2">
-        <v>310</v>
       </c>
       <c r="N40" t="s" s="2">
         <v>180</v>
@@ -5979,7 +5975,7 @@
         <v>80</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -5994,7 +5990,7 @@
         <v>139</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="AL40" t="s" s="2">
         <v>80</v>
@@ -6005,14 +6001,14 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
@@ -6034,10 +6030,10 @@
         <v>133</v>
       </c>
       <c r="L41" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="M41" t="s" s="2">
         <v>338</v>
-      </c>
-      <c r="M41" t="s" s="2">
-        <v>339</v>
       </c>
       <c r="N41" t="s" s="2">
         <v>180</v>
@@ -6092,7 +6088,7 @@
         <v>80</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6118,10 +6114,10 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6147,13 +6143,13 @@
         <v>193</v>
       </c>
       <c r="L42" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="M42" t="s" s="2">
         <v>342</v>
       </c>
-      <c r="M42" t="s" s="2">
+      <c r="N42" t="s" s="2">
         <v>343</v>
-      </c>
-      <c r="N42" t="s" s="2">
-        <v>344</v>
       </c>
       <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
@@ -6179,11 +6175,11 @@
         <v>80</v>
       </c>
       <c r="X42" t="s" s="2">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="Y42" s="2"/>
       <c r="Z42" t="s" s="2">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="AA42" t="s" s="2">
         <v>80</v>
@@ -6201,7 +6197,7 @@
         <v>80</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>78</v>
@@ -6216,7 +6212,7 @@
         <v>100</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="AL42" t="s" s="2">
         <v>80</v>
@@ -6227,14 +6223,14 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
@@ -6256,13 +6252,13 @@
         <v>193</v>
       </c>
       <c r="L43" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="M43" t="s" s="2">
         <v>350</v>
       </c>
-      <c r="M43" t="s" s="2">
+      <c r="N43" t="s" s="2">
         <v>351</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>352</v>
       </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
@@ -6291,11 +6287,11 @@
         <v>112</v>
       </c>
       <c r="Y43" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="Z43" t="s" s="2">
         <v>353</v>
       </c>
-      <c r="Z43" t="s" s="2">
-        <v>354</v>
-      </c>
       <c r="AA43" t="s" s="2">
         <v>80</v>
       </c>
@@ -6312,7 +6308,7 @@
         <v>80</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>88</v>
@@ -6333,19 +6329,19 @@
         <v>80</v>
       </c>
       <c r="AM43" t="s" s="2">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -6364,16 +6360,16 @@
         <v>80</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>307</v>
+        <v>149</v>
       </c>
       <c r="L44" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="M44" t="s" s="2">
         <v>358</v>
       </c>
-      <c r="M44" t="s" s="2">
+      <c r="N44" t="s" s="2">
         <v>359</v>
-      </c>
-      <c r="N44" t="s" s="2">
-        <v>360</v>
       </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
@@ -6423,7 +6419,7 @@
         <v>80</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>78</v>
@@ -6438,7 +6434,7 @@
         <v>100</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>80</v>
@@ -6449,10 +6445,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6478,10 +6474,10 @@
         <v>174</v>
       </c>
       <c r="L45" t="s" s="2">
+        <v>362</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>363</v>
-      </c>
-      <c r="M45" t="s" s="2">
-        <v>364</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6532,7 +6528,7 @@
         <v>80</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>78</v>
@@ -6553,15 +6549,15 @@
         <v>80</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6587,13 +6583,13 @@
         <v>108</v>
       </c>
       <c r="L46" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="M46" t="s" s="2">
         <v>367</v>
       </c>
-      <c r="M46" t="s" s="2">
+      <c r="N46" t="s" s="2">
         <v>368</v>
-      </c>
-      <c r="N46" t="s" s="2">
-        <v>369</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6622,11 +6618,11 @@
         <v>197</v>
       </c>
       <c r="Y46" t="s" s="2">
+        <v>369</v>
+      </c>
+      <c r="Z46" t="s" s="2">
         <v>370</v>
       </c>
-      <c r="Z46" t="s" s="2">
-        <v>371</v>
-      </c>
       <c r="AA46" t="s" s="2">
         <v>80</v>
       </c>
@@ -6643,7 +6639,7 @@
         <v>80</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
@@ -6669,10 +6665,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -6698,13 +6694,13 @@
         <v>193</v>
       </c>
       <c r="L47" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="M47" t="s" s="2">
         <v>373</v>
       </c>
-      <c r="M47" t="s" s="2">
+      <c r="N47" t="s" s="2">
         <v>374</v>
-      </c>
-      <c r="N47" t="s" s="2">
-        <v>375</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -6730,14 +6726,14 @@
         <v>80</v>
       </c>
       <c r="X47" t="s" s="2">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="Y47" t="s" s="2">
+        <v>375</v>
+      </c>
+      <c r="Z47" t="s" s="2">
         <v>376</v>
       </c>
-      <c r="Z47" t="s" s="2">
-        <v>377</v>
-      </c>
       <c r="AA47" t="s" s="2">
         <v>80</v>
       </c>
@@ -6754,7 +6750,7 @@
         <v>80</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>78</v>
@@ -6769,7 +6765,7 @@
         <v>100</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="AL47" t="s" s="2">
         <v>80</v>
@@ -6780,10 +6776,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -6809,13 +6805,13 @@
         <v>301</v>
       </c>
       <c r="L48" t="s" s="2">
+        <v>379</v>
+      </c>
+      <c r="M48" t="s" s="2">
         <v>380</v>
       </c>
-      <c r="M48" t="s" s="2">
+      <c r="N48" t="s" s="2">
         <v>381</v>
-      </c>
-      <c r="N48" t="s" s="2">
-        <v>382</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
@@ -6865,7 +6861,7 @@
         <v>80</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>78</v>

</xml_diff>

<commit_message>
demo-at: build triggered by rockphotog for commit e88b5c08d6854433102c5eacd3bb17d38164c0e9 e88b5c08d6854433102c5eacd3bb17d38164c0e9
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
+++ b/currentbuild/StructureDefinition-demo-at-allergy-intolerance.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.0</t>
+    <t>0.2.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -1123,10 +1123,10 @@
     <t>Clinical symptoms/signs associated with the Event</t>
   </si>
   <si>
-    <t>Clinical symptoms and/or signs that are observed or associated with the adverse reaction event.</t>
-  </si>
-  <si>
-    <t>Manifestation can be expressed as a single word, phrase or brief description. For example: nausea, rash or no reaction. It is preferable that manifestation should be coded with a terminology, where possible. The values entered here may be used to display on an application screen as part of a list of adverse reactions, as recommended in the UK NHS CUI guidelines.  Terminologies commonly used include, but are not limited to, SNOMED CT or ICD10.</t>
+    <t>Hvilken reaksjon pasienten har hatt.</t>
+  </si>
+  <si>
+    <t>Helse-NIM anbefaler KJ 7497 (Reaksjonstype) for koding av manifestasjon.</t>
   </si>
   <si>
     <t>Type of allergy or intolerance reaction expected to be used in MyHealth@EU</t>
@@ -1175,7 +1175,7 @@
     <t>Reaction severity</t>
   </si>
   <si>
-    <t>Clinical assessment of the severity of the reaction event as a whole, potentially considering multiple different manifestations.</t>
+    <t>Hvor alvorlig reaksjon pasienten har hatt.</t>
   </si>
   <si>
     <t>It is acknowledged that this assessment is very subjective. There may be some specific practice domains where objective scales have been applied. Objective scales can be included in this model as extensions.</t>
@@ -5670,7 +5670,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="38" hidden="true">
+    <row r="38">
       <c r="A38" t="s" s="2">
         <v>328</v>
       </c>
@@ -5689,7 +5689,7 @@
         <v>79</v>
       </c>
       <c r="H38" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I38" t="s" s="2">
         <v>80</v>
@@ -6221,7 +6221,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="43" hidden="true">
+    <row r="43">
       <c r="A43" t="s" s="2">
         <v>347</v>
       </c>
@@ -6240,7 +6240,7 @@
         <v>79</v>
       </c>
       <c r="H43" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I43" t="s" s="2">
         <v>80</v>
@@ -6552,7 +6552,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="46" hidden="true">
+    <row r="46">
       <c r="A46" t="s" s="2">
         <v>365</v>
       </c>
@@ -6571,7 +6571,7 @@
         <v>88</v>
       </c>
       <c r="H46" t="s" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I46" t="s" s="2">
         <v>80</v>

</xml_diff>